<commit_message>
Export and import assets, and give the sample company its assets from the workbook
An Assets sheet now exports with each asset's cost, depreciation
settings, depreciation to date and book value, and imports like the other
entity sheets. A row that names only a CRA class takes CRA's rate and
first-year share for its purchase date. Undoing an import also takes back
the assets it added.

The sample workbook carries six assets, from land owned before to a
label printer since sold, each linked to the purchase that bought it,
in place of the ones the sample company used to build in code.

The asset form's name and notes placeholders match the other forms, and
the fixed assets section of the calculations doc keeps to the maths.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ArgoBooks/Resources/SampleCompanyData.xlsx
+++ b/ArgoBooks/Resources/SampleCompanyData.xlsx
@@ -17,15 +17,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Adjustments" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Orders" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rental Inventory" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rental Records" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring Invoices" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Order Line Items" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lost Damaged" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Adjustments" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Orders" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rental Inventory" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rental Records" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring Invoices" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Order Line Items" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lost Damaged" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -5412,7 +5413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -6963,6 +6964,109 @@
       </c>
       <c r="J36" t="n">
         <v>1.12</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PUR-2025-036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2025-01-08</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Label Printer</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F37" t="n">
+        <v>60</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1260</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PUR-2025-037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2025-02-20</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Delivery Van</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>32000</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G38" t="n">
+        <v>33600</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Bank Transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PUR-2025-038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Staff Laptops</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F39" t="n">
+        <v>160</v>
+      </c>
+      <c r="G39" t="n">
+        <v>3360</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6976,8 +7080,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6987,547 +7108,355 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Product ID</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Location ID</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>In Stock</t>
+          <t>Purchase Date</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Reserved</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Reorder Point</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Unit Cost</t>
+          <t>Expense ID</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Useful Life (Years)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Rate %</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>CRA Class</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Disposed Date</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Disposal</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Sale Price</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INV-ITM-001</t>
+          <t>AST-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PRD-001</t>
+          <t>Storage lot</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>12</v>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2021-06-01</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G2" t="n">
-        <v>899</v>
+        <v>60000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>StraightLine</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Owned before the business started using Argo Books</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INV-ITM-002</t>
+          <t>AST-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PRD-002</t>
+          <t>Label printer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>6</v>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025-01-08</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1349</v>
+        <v>1200</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PUR-2025-036</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>DecliningBalance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Sold</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>700</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Replaced by a faster model</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INV-ITM-003</t>
+          <t>AST-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PRD-003</t>
+          <t>Delivery van</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>4</v>
+          <t>Vehicle</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2025-02-20</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" t="n">
-        <v>849</v>
+        <v>32000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PUR-2025-037</t>
+        </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>DecliningBalance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INV-ITM-004</t>
+          <t>AST-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PRD-004</t>
+          <t>Executive desk</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>8</v>
+          <t>FurnitureAndFixtures</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" t="n">
-        <v>699</v>
+        <v>3048.53</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PUR-2025-021</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>DecliningBalance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>INV-ITM-005</t>
+          <t>AST-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PRD-005</t>
+          <t>Staff laptops</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>5</v>
+          <t>ComputerEquipment</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1999</v>
+        <v>3200</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PUR-2025-038</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>DecliningBalance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>50</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>INV-ITM-006</t>
+          <t>AST-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PRD-006</t>
+          <t>Ergonomic office chairs</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>8</v>
+          <t>FurnitureAndFixtures</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" t="n">
-        <v>349</v>
+        <v>3048.51</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PUR-2025-022</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>INV-ITM-007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>PRD-007</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" t="n">
-        <v>8</v>
-      </c>
-      <c r="G8" t="n">
-        <v>149</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2025-12-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>INV-ITM-008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>PRD-008</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1195</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2025-12-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>INV-ITM-009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>PRD-009</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1515</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2025-12-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>INV-ITM-010</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>PRD-010</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" t="n">
-        <v>10</v>
-      </c>
-      <c r="G11" t="n">
-        <v>149</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2025-12-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>INV-ITM-011</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PRD-011</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>18</v>
-      </c>
-      <c r="E12" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" t="n">
-        <v>12</v>
-      </c>
-      <c r="G12" t="n">
-        <v>99</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2025-12-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>INV-ITM-012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PRD-012</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>20</v>
-      </c>
-      <c r="E13" t="n">
-        <v>5</v>
-      </c>
-      <c r="F13" t="n">
-        <v>12</v>
-      </c>
-      <c r="G13" t="n">
-        <v>89</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2025-12-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>INV-ITM-013</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PRD-013</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>LOC-001</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>14</v>
-      </c>
-      <c r="E14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G14" t="n">
-        <v>69</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>INV-ITM-014</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>PRD-006</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>LOC-002</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" t="n">
-        <v>349</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2025-12-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>INV-ITM-015</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PRD-007</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>LOC-002</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" t="n">
-        <v>149</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2025-12-15</t>
+          <t>DecliningBalance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -7542,7 +7471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -7553,397 +7482,547 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Inventory Item ID</t>
+          <t>Product ID</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Location ID</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>In Stock</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Previous Stock</t>
+          <t>Reserved</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>New Stock</t>
+          <t>Reorder Point</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Unit Cost</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Last Updated</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADJ-001</t>
+          <t>INV-ITM-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>INV-ITM-001</t>
+          <t>PRD-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Initial stock from PO-20001</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>899</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2025-01-05 10:00:00</t>
+          <t>2025-12-28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADJ-002</t>
+          <t>INV-ITM-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INV-ITM-004</t>
+          <t>PRD-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Initial stock from PO-20002</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1349</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2025-01-12 11:00:00</t>
+          <t>2025-12-20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADJ-003</t>
+          <t>INV-ITM-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>INV-ITM-006</t>
+          <t>PRD-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Initial stock from PO-20003</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>849</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2025-01-20 09:30:00</t>
+          <t>2025-12-15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADJ-004</t>
+          <t>INV-ITM-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INV-ITM-001</t>
+          <t>PRD-004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Remove</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" t="n">
-        <v>10</v>
-      </c>
       <c r="F5" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Sold to CUS-001</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>699</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2025-01-08 14:00:00</t>
+          <t>2025-12-28</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADJ-005</t>
+          <t>INV-ITM-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INV-ITM-004</t>
+          <t>PRD-005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Remove</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Sold to CUS-004</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1999</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2025-01-22 15:30:00</t>
+          <t>2025-12-22</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADJ-006</t>
+          <t>INV-ITM-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>INV-ITM-001</t>
+          <t>PRD-006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>16</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Restocked from PO-20011</t>
-        </is>
+        <v>6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>349</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2025-07-05 10:00:00</t>
+          <t>2025-12-25</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADJ-007</t>
+          <t>INV-ITM-007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>INV-ITM-005</t>
+          <t>PRD-007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Initial stock from PO-20007</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>149</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2025-04-10 11:00:00</t>
+          <t>2025-12-28</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADJ-008</t>
+          <t>INV-ITM-008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>INV-ITM-002</t>
+          <t>PRD-008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Initial stock from PO-20009</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1195</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2025-05-08 09:00:00</t>
+          <t>2025-12-18</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADJ-009</t>
+          <t>INV-ITM-009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>INV-ITM-013</t>
+          <t>PRD-009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Remove</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="n">
-        <v>15</v>
-      </c>
       <c r="F10" t="n">
-        <v>14</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Damaged during handling</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1515</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2025-08-15 16:00:00</t>
+          <t>2025-12-10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ADJ-010</t>
+          <t>INV-ITM-010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>INV-ITM-001</t>
+          <t>PRD-010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>LOC-001</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
         <v>10</v>
       </c>
-      <c r="F11" t="n">
-        <v>16</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Restocked from PO-20014</t>
-        </is>
+      <c r="G11" t="n">
+        <v>149</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2025-10-05 10:30:00</t>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>INV-ITM-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PRD-011</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LOC-001</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>12</v>
+      </c>
+      <c r="G12" t="n">
+        <v>99</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>INV-ITM-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PRD-012</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LOC-001</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" t="n">
+        <v>89</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>INV-ITM-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PRD-013</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LOC-001</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>69</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>INV-ITM-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PRD-006</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>LOC-002</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>349</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>INV-ITM-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PRD-007</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>LOC-002</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>149</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
         </is>
       </c>
     </row>
@@ -7958,7 +8037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -7969,267 +8048,397 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Supplier ID</t>
+          <t>Inventory Item ID</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Order Date</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Expected Date</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Previous Stock</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>New Stock</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PO-001</t>
+          <t>ADJ-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SUP-001</t>
+          <t>INV-ITM-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-01-02</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2025-01-09</t>
-        </is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>9731.68</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Received</t>
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Initial stock from PO-20001</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2025-01-05 10:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PO-002</t>
+          <t>ADJ-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUP-001</t>
+          <t>INV-ITM-004</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2025-01-17</t>
-        </is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>6053.34</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Received</t>
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Initial stock from PO-20002</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2025-01-12 11:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PO-003</t>
+          <t>ADJ-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SUP-004</t>
+          <t>INV-ITM-006</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-02-12</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2025-02-19</t>
-        </is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>3880.76</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Received</t>
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Initial stock from PO-20003</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2025-01-20 09:30:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PO-004</t>
+          <t>ADJ-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SUP-001</t>
+          <t>INV-ITM-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-04-08</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2025-04-15</t>
-        </is>
+          <t>Remove</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>8655.67</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Received</t>
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Sold to CUS-001</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2025-01-08 14:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PO-005</t>
+          <t>ADJ-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SUP-001</t>
+          <t>INV-ITM-004</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-07-02</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
+          <t>Remove</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>7785.34</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Received</t>
+        <v>8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Sold to CUS-004</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2025-01-22 15:30:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PO-006</t>
+          <t>ADJ-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SUP-001</t>
+          <t>INV-ITM-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-10-02</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2025-10-09</t>
-        </is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>5839.01</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Received</t>
+        <v>8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>16</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Restocked from PO-20011</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2025-07-05 10:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PO-007</t>
+          <t>ADJ-007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SUP-001</t>
+          <t>INV-ITM-005</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2025-12-27</t>
-        </is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>6491.75</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Sent</t>
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Initial stock from PO-20007</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2025-04-10 11:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PO-008</t>
+          <t>ADJ-008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SUP-007</t>
+          <t>INV-ITM-002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-01-05</t>
-        </is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>5514.26</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Draft</t>
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Initial stock from PO-20009</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2025-05-08 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ADJ-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>INV-ITM-013</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>15</v>
+      </c>
+      <c r="F10" t="n">
+        <v>14</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Damaged during handling</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2025-08-15 16:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ADJ-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>INV-ITM-001</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" t="n">
+        <v>16</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Restocked from PO-20014</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2025-10-05 10:30:00</t>
         </is>
       </c>
     </row>
@@ -8244,7 +8453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -8255,267 +8464,267 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Supplier ID</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Total Qty</t>
+          <t>Order Date</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Expected Date</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Rented</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Daily Rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Weekly Rate</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Monthly Rate</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Deposit</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
           <t>Status</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Product ID</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RNT-ITM-001</t>
+          <t>PO-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HD Projector</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D2" t="n">
-        <v>3</v>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-01-02</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025-01-09</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H2" t="n">
-        <v>800</v>
-      </c>
-      <c r="I2" t="n">
-        <v>250</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>PRD-041</t>
+        <v>9731.68</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Received</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RNT-ITM-002</t>
+          <t>PO-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Conference Room AV Kit</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-01-10</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025-01-17</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="n">
-        <v>150</v>
-      </c>
-      <c r="G3" t="n">
-        <v>600</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1800</v>
-      </c>
-      <c r="I3" t="n">
-        <v>500</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>PRD-042</t>
+        <v>6053.34</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Received</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RNT-ITM-003</t>
+          <t>PO-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Laptop Rental Unit</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" t="n">
-        <v>7</v>
+          <t>SUP-004</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-02-12</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2025-02-19</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" t="n">
-        <v>200</v>
-      </c>
-      <c r="H4" t="n">
-        <v>600</v>
-      </c>
-      <c r="I4" t="n">
-        <v>300</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>PRD-043</t>
+        <v>3880.76</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Received</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RNT-ITM-004</t>
+          <t>PO-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Portable PA System</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2</v>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2025-04-08</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2025-04-15</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="n">
-        <v>100</v>
-      </c>
-      <c r="G5" t="n">
-        <v>400</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I5" t="n">
-        <v>400</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>PRD-044</t>
+        <v>8655.67</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Received</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RNT-ITM-005</t>
+          <t>PO-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Display Monitor (Large)</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" t="n">
-        <v>4</v>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" t="n">
-        <v>40</v>
-      </c>
-      <c r="G6" t="n">
-        <v>160</v>
-      </c>
-      <c r="H6" t="n">
-        <v>500</v>
-      </c>
-      <c r="I6" t="n">
-        <v>200</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>PRD-045</t>
+        <v>7785.34</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PO-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-10-02</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025-10-09</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>5839.01</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PO-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>6491.75</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PO-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SUP-007</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>5514.26</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Draft</t>
         </is>
       </c>
     </row>
@@ -8530,7 +8739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -8541,524 +8750,267 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Customer ID</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rental Item ID</t>
+          <t>Total Qty</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Rate Type</t>
+          <t>Rented</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Rate Amount</t>
+          <t>Daily Rate</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Security Deposit</t>
+          <t>Weekly Rate</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Monthly Rate</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Due Date</t>
+          <t>Deposit</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Return Date</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Total Cost</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Paid</t>
+          <t>Product ID</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RNT-001</t>
+          <t>RNT-ITM-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CUS-003</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>RNT-ITM-001</t>
-        </is>
+          <t>HD Projector</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
       </c>
       <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
       <c r="F2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G2" t="n">
         <v>300</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
+        <v>800</v>
+      </c>
+      <c r="I2" t="n">
         <v>250</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2025-03-10</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2025-03-17</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2025-03-17</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>300</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>PRD-041</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RNT-002</t>
+          <t>RNT-ITM-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CUS-009</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>RNT-ITM-002</t>
-        </is>
+          <t>Conference Room AV Kit</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
+      <c r="E3" t="n">
+        <v>1</v>
       </c>
       <c r="F3" t="n">
+        <v>150</v>
+      </c>
+      <c r="G3" t="n">
         <v>600</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I3" t="n">
         <v>500</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2025-05-05</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2025-05-12</t>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2025-05-11</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>600</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>PRD-042</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RNT-003</t>
+          <t>RNT-ITM-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CUS-007</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>RNT-ITM-003</t>
-        </is>
+          <t>Laptop Rental Unit</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
       </c>
       <c r="D4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
       <c r="F4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" t="n">
         <v>200</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
+        <v>600</v>
+      </c>
+      <c r="I4" t="n">
         <v>300</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2025-07-15</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2025-07-22</t>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2025-07-22</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>600</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>PRD-043</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RNT-004</t>
+          <t>RNT-ITM-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CUS-011</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>RNT-ITM-001</t>
-        </is>
+          <t>Portable PA System</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
       </c>
       <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
       <c r="F5" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>250</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2025-09-20</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2025-09-27</t>
-        </is>
+        <v>400</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I5" t="n">
+        <v>400</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2025-09-27</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>300</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>PRD-044</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RNT-005</t>
+          <t>RNT-ITM-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CUS-015</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>RNT-ITM-004</t>
-        </is>
+          <t>Display Monitor (Large)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>400</v>
+        <v>40</v>
       </c>
       <c r="G6" t="n">
-        <v>400</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2025-10-10</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2025-10-17</t>
-        </is>
+        <v>160</v>
+      </c>
+      <c r="H6" t="n">
+        <v>500</v>
+      </c>
+      <c r="I6" t="n">
+        <v>200</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>400</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>RNT-006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CUS-003</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>RNT-ITM-005</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>160</v>
-      </c>
-      <c r="G7" t="n">
-        <v>200</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2025-12-15</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>320</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>RNT-007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>CUS-011</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>RNT-ITM-001</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G8" t="n">
-        <v>250</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2025-12-26</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-01-02</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>300</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>RNT-008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CUS-009</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>RNT-ITM-003</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>200</v>
-      </c>
-      <c r="G9" t="n">
-        <v>300</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2025-12-28</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-01-04</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>400</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>PRD-045</t>
         </is>
       </c>
     </row>
@@ -9073,7 +9025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -9089,167 +9041,519 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Rental Item ID</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Frequency</t>
+          <t>Rate Type</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Next Date</t>
+          <t>Rate Amount</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Security Deposit</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Return Date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Total Cost</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Paid</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REC-INV-001</t>
+          <t>RNT-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CUS-002</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>800</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Monthly IT Support Contract</t>
-        </is>
+          <t>CUS-003</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>RNT-ITM-001</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-01-02</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>300</v>
+      </c>
+      <c r="G2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2025-03-10</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2025-03-17</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2025-03-17</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>300</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REC-INV-002</t>
+          <t>RNT-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CUS-001</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>528</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CloudOffice Business Premium (2 users)</t>
-        </is>
+          <t>CUS-009</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RNT-ITM-002</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>600</v>
+      </c>
+      <c r="G3" t="n">
+        <v>500</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2025-05-05</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2025-05-11</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>600</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REC-INV-003</t>
+          <t>RNT-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CUS-006</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Quarterly Network Maintenance</t>
-        </is>
+          <t>CUS-007</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RNT-ITM-003</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-01-25</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>200</v>
+      </c>
+      <c r="G4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2025-07-15</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>600</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REC-INV-004</t>
+          <t>RNT-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CUS-012</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2400</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Annual Support Agreement</t>
-        </is>
+          <t>CUS-011</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>RNT-ITM-001</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Annually</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>300</v>
+      </c>
+      <c r="G5" t="n">
+        <v>250</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2025-09-27</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2025-09-27</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>300</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RNT-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CUS-015</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>RNT-ITM-004</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>400</v>
+      </c>
+      <c r="G6" t="n">
+        <v>400</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2025-10-10</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2025-10-17</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>400</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RNT-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CUS-003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>RNT-ITM-005</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>160</v>
+      </c>
+      <c r="G7" t="n">
+        <v>200</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>320</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RNT-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CUS-011</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RNT-ITM-001</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G8" t="n">
+        <v>250</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>300</v>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RNT-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CUS-009</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RNT-ITM-003</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>200</v>
+      </c>
+      <c r="G9" t="n">
+        <v>300</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>400</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -9259,6 +9563,197 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Customer ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Frequency</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Next Date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REC-INV-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CUS-002</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>800</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Monthly IT Support Contract</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REC-INV-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CUS-001</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>528</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CloudOffice Business Premium (2 users)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REC-INV-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CUS-006</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Quarterly Network Maintenance</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REC-INV-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CUS-012</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Annual Support Agreement</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Annually</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9726,332 +10221,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Original Transaction ID</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Return Type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Customer ID</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Supplier ID</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Return Date</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Refund Amount</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Restocking Fee</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Reason</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>RET-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PUR-2025-005</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>SUP-004</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>SecureGate MX68 Firewall</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>46025.88398792824</v>
-      </c>
-      <c r="I2" t="n">
-        <v>411.1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Defective</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>RET-002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PUR-2025-008</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>SUP-004</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>NetSwitch 1000-24T</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>46035.88398792824</v>
-      </c>
-      <c r="I3" t="n">
-        <v>170.61</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Not as described</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>RET-003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PUR-2025-010</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>SUP-002</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PeripheralPro Bundle</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>46045.88398792824</v>
-      </c>
-      <c r="I4" t="n">
-        <v>89.98999999999999</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Changed mind</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>RET-004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SAL-2025-013</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>CUS-006</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ByteForge ThinkPad T14</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>46030.88398792824</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1299</v>
-      </c>
-      <c r="J5" t="n">
-        <v>50</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Defective</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>RET-005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SAL-2025-006</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CUS-004</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>WorkStation 7010 Desktop</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>46040.88398792824</v>
-      </c>
-      <c r="I6" t="n">
-        <v>899</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Changed mind</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -10585,6 +10754,332 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Original Transaction ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Return Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Customer ID</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Supplier ID</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Return Date</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Refund Amount</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Restocking Fee</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RET-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PUR-2025-005</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SUP-004</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SecureGate MX68 Firewall</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>46025.88398792824</v>
+      </c>
+      <c r="I2" t="n">
+        <v>411.1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Defective</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RET-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PUR-2025-008</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SUP-004</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NetSwitch 1000-24T</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>46035.88398792824</v>
+      </c>
+      <c r="I3" t="n">
+        <v>170.61</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Not as described</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RET-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PUR-2025-010</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SUP-002</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PeripheralPro Bundle</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>46045.88398792824</v>
+      </c>
+      <c r="I4" t="n">
+        <v>89.98999999999999</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Changed mind</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RET-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SAL-2025-013</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CUS-006</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ByteForge ThinkPad T14</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>46030.88398792824</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1299</v>
+      </c>
+      <c r="J5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Defective</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RET-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SAL-2025-006</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CUS-004</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>WorkStation 7010 Desktop</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>46040.88398792824</v>
+      </c>
+      <c r="I6" t="n">
+        <v>899</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Changed mind</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
@@ -10769,7 +11264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -11346,6 +11841,33 @@
         </is>
       </c>
       <c r="F17" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CAT-PUR-006</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Equipment and Vehicles</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Vehicles, furniture and equipment kept for years</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
@@ -11362,7 +11884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8.7265625" customWidth="1" min="2" max="2"/>
@@ -13908,6 +14430,132 @@
       </c>
       <c r="L46" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PRD-046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Delivery Van</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>EXP-VAN</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Cargo van for customer deliveries</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>CAT-PUR-006</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Equipment and Vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PRD-047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Staff Laptops</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>EXP-STAFF-LAPTOPS</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Laptops for staff to use, not for resale</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>CAT-PUR-006</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Equipment and Vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PRD-048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Label Printer</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>EXP-LABEL-PRINTER</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Thermal label printer for shipping</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>CAT-PUR-006</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Equipment and Vehicles</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Count what a sold asset brings in as profit on the dashboard
The dashboard already counts an asset's purchase as an expense in full, so its sale price now comes back into Net Profit, Profit Margin and Profit Over Time on the day it sold. It stays out of revenue, since it is not a sale to a customer.

The sample company's van is now a used one at $7,500, so its purchase no longer dwarfs every other day on the charts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ArgoBooks/Resources/SampleCompanyData.xlsx
+++ b/ArgoBooks/Resources/SampleCompanyData.xlsx
@@ -7019,13 +7019,13 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>32000</v>
+        <v>7500</v>
       </c>
       <c r="F38" t="n">
-        <v>1600</v>
+        <v>375</v>
       </c>
       <c r="G38" t="n">
-        <v>33600</v>
+        <v>7875</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -7288,7 +7288,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Delivery van</t>
+          <t>Used delivery van</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -7302,7 +7302,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>32000</v>
+        <v>7500</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Cargo van for customer deliveries</t>
+          <t>Used cargo van for customer deliveries</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">

</xml_diff>

<commit_message>
Keep the sample company's forecast in profit
The forecast for next month always reads the sample data's February, which a delivery van and a stationery order pushed into a loss. They now fall in July and April.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ArgoBooks/Resources/SampleCompanyData.xlsx
+++ b/ArgoBooks/Resources/SampleCompanyData.xlsx
@@ -6244,7 +6244,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2025-02-25</t>
+          <t>2025-04-22</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2025-02-20</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2025-02-20</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E4" t="n">

</xml_diff>